<commit_message>
Admin Update - 2026-10-02T00:52:15.185Z
</commit_message>
<xml_diff>
--- a/links_utm_stellantis.xlsx
+++ b/links_utm_stellantis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luism\Documents\landing_stellantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A6E529-FA9D-4561-A7AC-09F9AFF9C43D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3151055A-2850-4A45-ABA4-422EF674B3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Enlaces UTM'!$A$1:$H$73</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -1178,7 +1178,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:H73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.796875" customWidth="1"/>
     <col min="2" max="2" width="28.796875" customWidth="1"/>
@@ -1189,7 +1189,7 @@
     <col min="8" max="8" width="80.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1215,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1241,7 +1241,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1319,7 +1319,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1527,7 +1527,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>63</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>63</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -1761,7 +1761,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1787,7 +1787,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>63</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>63</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>94</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>94</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>94</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>94</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>94</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>94</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>94</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>94</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>94</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>94</v>
       </c>
@@ -2099,7 +2099,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>94</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>94</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>94</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>94</v>
       </c>
@@ -2203,7 +2203,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>94</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>145</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>145</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>145</v>
       </c>
@@ -2307,7 +2307,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>145</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>145</v>
       </c>
@@ -2359,7 +2359,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>145</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>145</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>145</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>145</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>176</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>176</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>176</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>176</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>176</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>176</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>176</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>176</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>176</v>
       </c>
@@ -2697,7 +2697,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>176</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>176</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>176</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>176</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>176</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>176</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>176</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>176</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>176</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>237</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>237</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>237</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>248</v>
       </c>
@@ -3035,7 +3035,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>248</v>
       </c>
@@ -3061,7 +3061,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>248</v>
       </c>
@@ -3091,8 +3091,7 @@
   <autoFilter ref="A1:H73" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="1">
       <filters>
-        <filter val="Dodge Attitude SXT"/>
-        <filter val="Leapmotor B10"/>
+        <filter val="Jeep Renegade"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>